<commit_message>
Adiciona pipeline inicial de analise de repelencia em R
</commit_message>
<xml_diff>
--- a/dados/dados_brutos.xlsx
+++ b/dados/dados_brutos.xlsx
@@ -18,10 +18,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0000000"/>
-  </numFmts>
-  <fonts count="5">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,17 +29,6 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00000000"/>
-    </font>
-    <font>
-      <color rgb="00008000"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00666666"/>
-    </font>
-    <font>
-      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="3">
@@ -53,11 +40,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009DC3E6"/>
+        <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -65,35 +52,19 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <bottom style="medium">
-        <color rgb="005B9BD5"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -170,65 +141,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>OpenAI</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Rotulo transcrito literalmente da primeira coluna da imagem enviada.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Contagem de individuos no lado tratado em cada repeticao.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Contagem de individuos no lado nao tratado em cada repeticao.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabelaDadosBrutos" displayName="TabelaDadosBrutos" ref="A1:E13" headerRowCount="1">
-  <autoFilter ref="A1:E13"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="identificador_original"/>
-    <tableColumn id="2" name="tempo_h"/>
-    <tableColumn id="3" name="repeticao"/>
-    <tableColumn id="4" name="tratado"/>
-    <tableColumn id="5" name="nao_tratado"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TabelaResumoOriginal" displayName="TabelaResumoOriginal" ref="A1:K7" headerRowCount="1">
-  <autoFilter ref="A1:K7"/>
-  <tableColumns count="11">
-    <tableColumn id="1" name="identificador_original"/>
-    <tableColumn id="2" name="tempo_h"/>
-    <tableColumn id="3" name="total_tratado"/>
-    <tableColumn id="4" name="total_nao_tratado"/>
-    <tableColumn id="5" name="raiz_total_tratado"/>
-    <tableColumn id="6" name="raiz_total_nao_tratado"/>
-    <tableColumn id="7" name="desvio_tratado"/>
-    <tableColumn id="8" name="desvio_nao_tratado"/>
-    <tableColumn id="9" name="erro_tratado"/>
-    <tableColumn id="10" name="erro_nao_tratado"/>
-    <tableColumn id="11" name="anotacao_estatistica_original"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -520,277 +432,207 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>identificador_original</t>
+          <t>tempo_h</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>tempo_h</t>
+          <t>repeticao</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>repeticao</t>
+          <t>tratado</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>tratado</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
           <t>nao_tratado</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>aza</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="3" t="n">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
         <v>25</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="D2" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>aza</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="3" t="n">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="C3" t="n">
         <v>23</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="D3" t="n">
         <v>38</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>aza</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3" t="n">
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
         <v>26</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="D4" t="n">
         <v>34</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>aza</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="B5" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="C5" t="n">
         <v>24</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="D5" t="n">
         <v>43</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
+      <c r="A6" t="n">
         <v>6</v>
       </c>
-      <c r="C6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="3" t="n">
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
         <v>26</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="D6" t="n">
         <v>38</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="B7" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="C7" t="n">
         <v>25</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="D7" t="n">
         <v>43</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
+      <c r="A8" t="n">
         <v>12</v>
       </c>
-      <c r="C8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="3" t="n">
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
         <v>26</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="D8" t="n">
         <v>38</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
+      <c r="A9" t="n">
         <v>12</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="B9" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="C9" t="n">
         <v>25</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="D9" t="n">
         <v>43</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
+      <c r="A10" t="n">
         <v>24</v>
       </c>
-      <c r="C10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="3" t="n">
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
         <v>26</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="D10" t="n">
         <v>43</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
+      <c r="A11" t="n">
         <v>24</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="B11" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="C11" t="n">
         <v>25</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="D11" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
+      <c r="A12" t="n">
         <v>48</v>
       </c>
-      <c r="C12" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="3" t="n">
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
         <v>27</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="D12" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
+      <c r="A13" t="n">
         <v>48</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="B13" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="C13" t="n">
         <v>25</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="D13" t="n">
         <v>43</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -800,308 +642,272 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>identificador_original</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>tempo_h</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>total_tratado</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>total_nao_tratado</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>raiz_total_tratado</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>raiz_total_nao_tratado</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>desvio_tratado</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>desvio_nao_tratado</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>tratado_total</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>nao_tratado_total</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>raiz_tratado</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>raiz_nao_tratado</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>desvio_pa_tratado</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>desvio_pa_nao_tratado</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>erro_tratado</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>erro_nao_tratado</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
-        <is>
-          <t>anotacao_estatistica_original</t>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>anotacao_original</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>aza</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="3" t="n">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
         <v>48</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="C2" t="n">
         <v>71</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="D2" t="n">
         <v>6.9282032</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="E2" t="n">
         <v>8.426149799999999</v>
       </c>
-      <c r="G2" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="5" t="n">
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
         <v>2.5</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="H2" t="n">
         <v>0.1443376</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="I2" t="n">
         <v>0.2966954</v>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>p valor &lt; 0,001</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>aza</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
+      <c r="A3" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="B3" t="n">
         <v>50</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="C3" t="n">
         <v>77</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="D3" t="n">
         <v>7.0710678</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="E3" t="n">
         <v>8.7749644</v>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="5" t="n">
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
         <v>4.5</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="H3" t="n">
         <v>0.1414214</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="I3" t="n">
         <v>0.5128226</v>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>p valor &lt; 0,001</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
+      <c r="A4" t="n">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="B4" t="n">
         <v>51</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="C4" t="n">
         <v>81</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="D4" t="n">
         <v>7.1414284</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="E4" t="n">
         <v>9</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="F4" t="n">
         <v>0.5</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="G4" t="n">
         <v>2.5</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="H4" t="n">
         <v>0.07001400000000001</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="I4" t="n">
         <v>0.2777778</v>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>p valor &lt; 0,0001</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
+      <c r="A5" t="n">
         <v>12</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="B5" t="n">
         <v>51</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="C5" t="n">
         <v>81</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="D5" t="n">
         <v>7.1414284</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="E5" t="n">
         <v>9</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="F5" t="n">
         <v>0.5</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="G5" t="n">
         <v>2.5</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="H5" t="n">
         <v>0.07001400000000001</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="I5" t="n">
         <v>0.2777778</v>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>p valor &lt; 0,001</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
+      <c r="A6" t="n">
         <v>24</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="B6" t="n">
         <v>51</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="C6" t="n">
         <v>82</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="D6" t="n">
         <v>7.1414284</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="E6" t="n">
         <v>9.055385100000001</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="F6" t="n">
         <v>0.5</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="G6" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="H6" t="n">
         <v>0.07001400000000001</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="I6" t="n">
         <v>0.2208631</v>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>X2 = 0,0038</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>ML4</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
+      <c r="A7" t="n">
         <v>48</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="B7" t="n">
         <v>52</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="C7" t="n">
         <v>82</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="D7" t="n">
         <v>7.2111026</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="E7" t="n">
         <v>9.055385100000001</v>
       </c>
-      <c r="G7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="5" t="n">
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="H7" t="n">
         <v>0.138675</v>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="I7" t="n">
         <v>0.2208631</v>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>X2 = 0,2159</t>
         </is>
@@ -1109,9 +915,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
@@ -1121,94 +924,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Observacao</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Origem</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Valores transcritos da imagem enviada na conversa.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Formato recomendado para R</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Use a aba dados_brutos. Cada linha corresponde a uma repeticao em um tempo.</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Uso recomendado</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>A aba dados_brutos deve ser usada pelos scripts R.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Repeticoes 3R e 4R</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Aparecem vazias na imagem; por isso nao foram inventadas nem preenchidas.</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Limite metodologico</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Foi informado que cada repeticao acompanha os mesmos 30 acaros ao longo do tempo. Entretanto, varias linhas somam mais de 30 (tratado + nao_tratado). Isso indica que estes valores podem ser agregados/cumulativos e nao contagens instantaneas simples por arena.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Identificador original</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>A imagem mostra "aza" em 1 h e 3 h, e "ML4" em 6, 12, 24 e 48 h; os rotulos foram preservados literalmente.</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Consequencia</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Os scripts 03 e 04 devem ser interpretados como analises de frequencias agregadas, nao como modelo final de medidas repetidas.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Resumo original</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>A aba resumo_original preserva totais, raiz do total, desvio, erro e a anotacao estatistica exibida na imagem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Cuidado estatistico</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>A anotacao X2/p-valor foi preservada como texto e nao foi reinterpretada neste arquivo.</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Metodo antigo</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>A imagem do SAS mostra PROC FREQ / Chi-Square Test for Equal Proportions; o script 04 reproduz essa logica em R.</t>
         </is>
       </c>
     </row>

</xml_diff>